<commit_message>
Publish PR preview pr-54
</commit_message>
<xml_diff>
--- a/pr-preview/pr-54/obyvak-skladba-materialu.xlsx
+++ b/pr-preview/pr-54/obyvak-skladba-materialu.xlsx
@@ -1645,26 +1645,26 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Latový rošt</t>
+          <t>Rošt kastlíku</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Dřevěné latě</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40 mm</t>
+          <t>Profil CD 60×27</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Rigips R-CD 27/60/27</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>60×40 @ 625</t>
+          <t>60×27 @ 625</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1673,26 +1673,26 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>12 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>19.7</v>
+        <v>19.1</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>45</v>
+        <v>29.21</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>885</v>
+        <v>557</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>orientační řezivo KVH/latě CZ e-shopy</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>32 prvků (svislé + spodní).</t>
+          <t>32 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Drop CD → latový rošt</t>
+          <t>Drop CD → svislý CD</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2183,7 +2183,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16627</v>
+        <v>16299</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2218,9 +2218,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2418,11 +2419,11 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>60×27 @ 625</t>
+          <t>kuchyň 625 svisle + dořez; obývák 1000 + dořez</t>
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>109.4</v>
+        <v>101.8</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -2435,13 +2436,13 @@
         </is>
       </c>
       <c r="I4" s="9" t="n">
-        <v>120.3</v>
+        <v>111.9</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>3515</v>
+        <v>3270</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -2450,7 +2451,7 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>UW detaily dle montáže — v modelu jako CD.</t>
+          <t>Lišty pod spárou: kuchyň 2000 mm, obývák 1250 a 2500 mm, na CD. UW v modelu jako CD.</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2482,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -2494,13 +2495,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>47.5</v>
+        <v>37.8</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>22667</v>
+        <v>18031</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -2705,7 +2706,7 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>28105</v>
+        <v>23223</v>
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -3272,7 +3273,7 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>219.7</v>
+        <v>229.4</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -3285,13 +3286,13 @@
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>241.7</v>
+        <v>252.4</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7060</v>
+        <v>7372</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -3443,7 +3444,7 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3456,13 +3457,13 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>47.5</v>
+        <v>37.8</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>22667</v>
+        <v>18031</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -3500,7 +3501,7 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>33.07</v>
+        <v>33.09</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -3513,7 +3514,7 @@
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>36.38</v>
+        <v>36.4</v>
       </c>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
@@ -3524,64 +3525,64 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.63 m³.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="7" t="n">
+          <t>Plenum 27.64 + kastlík 1.80 + štíty 3.65 m³.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Řezivo</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Latě 60×40</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>60×40</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>UD 28×27</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>UD profil</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Rigips UD (obvod kastlíku)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>28×27</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>12 %</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>885</v>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>orientační řezivo KVH/latě CZ e-shopy</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>Kastlík.</t>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>29.21</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>336</v>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3902,7 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="16" t="n">
-        <v>105702</v>
+        <v>100828</v>
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>

</xml_diff>